<commit_message>
fix(v1.3): add chip and crew prices to authoritative Excel workbook
</commit_message>
<xml_diff>
--- a/tools/data_source/bridge_data.xlsx
+++ b/tools/data_source/bridge_data.xlsx
@@ -259,157 +259,244 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="65" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="6" t="str">
-        <x:v>chip_id</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>display_name</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
-        <x:v>rarity</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="E1" s="6" t="str">
-        <x:v>icon_path</x:v>
-      </x:c>
-      <x:c r="F1" s="6" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" t="str">
-        <x:v>chip_fire_01</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>火控强化 I</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>COMMON</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>全舰武器伤害提高</x:v>
-      </x:c>
-      <x:c r="E2" t="str"/>
-      <x:c r="F2" t="str">
-        <x:v>[{"stat":"weapon_damage","operation":"PERCENT_ADD","value":0.15,"target_filter":"ALL"}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" t="str">
-        <x:v>chip_energy_01</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>反应堆优化</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>COMMON</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>能源输出提高</x:v>
-      </x:c>
-      <x:c r="E3" t="str"/>
-      <x:c r="F3" t="str">
-        <x:v>[{"stat":"energy_output","operation":"PERCENT_ADD","value":0.2,"target_filter":"ALL"}]</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>chip_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rarity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>icon_path</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>chip_fire_01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>火控强化 I</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>全舰武器伤害提高</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>[{"stat":"weapon_damage","operation":"PERCENT_ADD","value":0.15,"target_filter":"ALL"}]</t>
+        </is>
+      </c>
+      <c r="G2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chip_energy_01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>反应堆优化</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>能源输出提高</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[{"stat":"energy_output","operation":"PERCENT_ADD","value":0.2,"target_filter":"ALL"}]</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="65" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="6" t="str">
-        <x:v>crew_id</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>display_name</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
-        <x:v>race</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>rarity</x:v>
-      </x:c>
-      <x:c r="E1" s="6" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="F1" s="6" t="str">
-        <x:v>portrait_path</x:v>
-      </x:c>
-      <x:c r="G1" s="6" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" t="str">
-        <x:v>crew_human_01</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>莱恩</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>HUMAN</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>COMMON</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>改善武器射程</x:v>
-      </x:c>
-      <x:c r="F2" t="str"/>
-      <x:c r="G2" t="str">
-        <x:v>[{"stat":"weapon_range","operation":"PERCENT_ADD","value":0.08,"target_filter":"ALL"}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" t="str">
-        <x:v>crew_machine_01</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>AX-07</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>MACHINE</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>UNCOMMON</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>提高武器伤害</x:v>
-      </x:c>
-      <x:c r="F3" t="str"/>
-      <x:c r="G3" t="str">
-        <x:v>[{"stat":"weapon_damage","operation":"PERCENT_ADD","value":0.12,"target_filter":"ALL"}]</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>crew_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rarity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>portrait_path</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>crew_human_01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>莱恩</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HUMAN</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>改善武器射程</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>[{"stat":"weapon_range","operation":"PERCENT_ADD","value":0.08,"target_filter":"ALL"}]</t>
+        </is>
+      </c>
+      <c r="H2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>crew_machine_01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AX-07</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MACHINE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>提高武器伤害</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[{"stat":"weapon_damage","operation":"PERCENT_ADD","value":0.12,"target_filter":"ALL"}]</t>
+        </is>
+      </c>
+      <c r="H3">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>